<commit_message>
rivosto tutto il programma e dovrebbe essere tutto corretto
</commit_message>
<xml_diff>
--- a/Tomoscan_pso_interlaced/risultati_corput_N32_K4_PSO20000.xlsx
+++ b/Tomoscan_pso_interlaced/risultati_corput_N32_K4_PSO20000.xlsx
@@ -8,9 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="MOD360" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UNWRAPPED" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="COUNTS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DELTA_THETA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="UNWRAPPED_ACQ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="COUNTS_PSO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DELTA_THETA_PSO" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,7 +422,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>target_deg</t>
+          <t>target_deg_mod360</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -2250,7 +2250,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>target_deg</t>
+          <t>target_deg_unwrapped_acq</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -4078,7 +4078,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>theta_unwrapped_deg</t>
+          <t>theta_monotonic_deg</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">

</xml_diff>